<commit_message>
Add functionality to insert and delete rows in Excel files and create a new sheet with sales data and a bar chart
</commit_message>
<xml_diff>
--- a/Book/chapter14/multiplication.xlsx
+++ b/Book/chapter14/multiplication.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,83 +453,83 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D3" t="n">
-        <v>6</v>
-      </c>
-      <c r="E3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F3" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D4" t="n">
-        <v>9</v>
-      </c>
-      <c r="E4" t="n">
-        <v>12</v>
-      </c>
-      <c r="F4" t="n">
-        <v>15</v>
-      </c>
-    </row>
     <row r="5">
       <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="n">
         <v>8</v>
       </c>
-      <c r="D5" t="n">
-        <v>12</v>
-      </c>
-      <c r="E5" t="n">
-        <v>16</v>
-      </c>
       <c r="F5" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" t="n">
+        <v>9</v>
+      </c>
+      <c r="E6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F6" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D7" t="n">
+        <v>12</v>
+      </c>
+      <c r="E7" t="n">
+        <v>16</v>
+      </c>
+      <c r="F7" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B8" t="n">
         <v>5</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C8" t="n">
         <v>10</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D8" t="n">
         <v>15</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E8" t="n">
         <v>20</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F8" t="n">
         <v>25</v>
       </c>
     </row>

</xml_diff>